<commit_message>
Sample proposal v2: full 16-page Technical Volume + complete deck/cost + canvas templates
- Technical Volume expanded to a genuine full-length SBIR volume (15 numbered
  sections + 2 appendices, 12pt/1.5): added §2.6 Model Architecture, §2.7
  Robustness, expanded §1 (operational requirements + why-now), §14 IP & Data
  Rights, §15 Broader Impacts, 2nd figure (inference pipeline), more tables.
  Authoritative page count (pdfjs-dist): 16 pages docx + pdf.
- Commercialization: 5 complete slides. Cost Volume: 2 tabs (Direct-Labor detail
  + Budget Summary), currency + subtotals, $150,000 total.
- docs/sample-proposal/canvas/*.canvas.json — each deliverable's source
  CanvasDocument saved as a reusable example template.
- README reframed as canonical example outputs/templates.

Generated by frontend/scripts/gen-sample-proposal.mts (real exporters). tsc 0.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WpKLE6LTPMraFbTacbbBV
</commit_message>
<xml_diff>
--- a/docs/sample-proposal/Aerivio_Cost_Volume.xlsx
+++ b/docs/sample-proposal/Aerivio_Cost_Volume.xlsx
@@ -4,17 +4,79 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Phase I Budget" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Direct Labor" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Budget Summary" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Phase I Budget'!$A1:$C8</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Direct Labor'!$A1:$D5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Budget Summary'!$A1:$C9</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="43">
+  <si>
+    <t>Role / Name</t>
+  </si>
+  <si>
+    <t>Hourly rate</t>
+  </si>
+  <si>
+    <t>Hours</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Principal Investigator — Dr. Ellison</t>
+  </si>
+  <si>
+    <t>95</t>
+  </si>
+  <si>
+    <t>360</t>
+  </si>
+  <si>
+    <t>34200</t>
+  </si>
+  <si>
+    <t>Senior Systems Engineer — Reyes</t>
+  </si>
+  <si>
+    <t>78</t>
+  </si>
+  <si>
+    <t>440</t>
+  </si>
+  <si>
+    <t>34320</t>
+  </si>
+  <si>
+    <t>ML Engineer — Nandakumar</t>
+  </si>
+  <si>
+    <t>62</t>
+  </si>
+  <si>
+    <t>312</t>
+  </si>
+  <si>
+    <t>19340</t>
+  </si>
+  <si>
+    <t>Subtotal — Direct Labor</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>1112</t>
+  </si>
+  <si>
+    <t>87860</t>
+  </si>
   <si>
     <t>Cost Category</t>
   </si>
@@ -22,16 +84,10 @@
     <t>Basis</t>
   </si>
   <si>
-    <t>Amount</t>
-  </si>
-  <si>
     <t>Direct Labor</t>
   </si>
   <si>
-    <t>PI 0.30 FTE + 2 engineers</t>
-  </si>
-  <si>
-    <t>88000</t>
+    <t>PI + 2 engineers (1,112 hrs)</t>
   </si>
   <si>
     <t>Fringe Benefits</t>
@@ -40,13 +96,13 @@
     <t>25% of direct labor</t>
   </si>
   <si>
-    <t>22000</t>
+    <t>21965</t>
   </si>
   <si>
     <t>Materials &amp; Supplies</t>
   </si>
   <si>
-    <t>Edge compute modules, hydrophones</t>
+    <t>Edge compute kits (×2), hydrophones</t>
   </si>
   <si>
     <t>8000</t>
@@ -64,25 +120,28 @@
     <t>Consultant</t>
   </si>
   <si>
-    <t>Acoustics SME (40 hrs)</t>
-  </si>
-  <si>
-    <t>12000</t>
+    <t>Acoustics SME (40 hrs @ $150)</t>
+  </si>
+  <si>
+    <t>6000</t>
+  </si>
+  <si>
+    <t>Subtotal — Direct Costs</t>
+  </si>
+  <si>
+    <t>127825</t>
   </si>
   <si>
     <t>Indirect (Overhead)</t>
   </si>
   <si>
-    <t>18% modified total</t>
-  </si>
-  <si>
-    <t>16000</t>
+    <t>17.3% of modified total</t>
+  </si>
+  <si>
+    <t>22175</t>
   </si>
   <si>
     <t>TOTAL</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>150000</t>
@@ -108,7 +167,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -118,6 +177,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE0E0E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFe0e7ff"/>
       </patternFill>
     </fill>
     <fill>
@@ -145,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -153,10 +217,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -501,100 +571,200 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="36" customWidth="1"/>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="4" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="37" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>20</v>
+      <c r="C7" s="3" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>23</v>
+      <c r="A8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>